<commit_message>
chore: refresh Batch Start to Picked date (2026-09-22T19:00Z)
</commit_message>
<xml_diff>
--- a/Batch_Start_to_Picked_date.xlsx
+++ b/Batch_Start_to_Picked_date.xlsx
@@ -1646,10 +1646,10 @@
         <v>46303</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E47" s="3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: refresh Batch Start to Picked date (2026-09-23T19:07Z)
</commit_message>
<xml_diff>
--- a/Batch_Start_to_Picked_date.xlsx
+++ b/Batch_Start_to_Picked_date.xlsx
@@ -1864,13 +1864,13 @@
         <v>46242</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>121</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>6</v>
@@ -1926,10 +1926,10 @@
         <v>46303</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="G47" s="3" t="n">
         <v>0</v>

</xml_diff>